<commit_message>
Re-scrape with correct Apify actor - real prices for June 24
</commit_message>
<xml_diff>
--- a/kapiva_data_2026-06-24.xlsx
+++ b/kapiva_data_2026-06-24.xlsx
@@ -486,17 +486,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kapiva Liver Care Juice (1L) | Anti-oxidant Rich Supplement With 5 Ayurvedic Herbs | Supports Fatty Liver Management &amp; Detox</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>500</v>
+        <v>628</v>
       </c>
       <c r="F2" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="G2" t="n">
-        <v>1624</v>
+        <v>1641</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -532,17 +532,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kapiva Shilajit/Shilajeet Gold Resin</t>
+          <t>Kapiva Shilajit/Shilajeet Gold Resin - 20g | 500mg/Serving | 40 Servings | Boost Muscle Growth &amp; Stamina | Contains 24 Carat Gold | 100% Ayurvedic</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>500</v>
+        <v>1254</v>
       </c>
       <c r="F3" t="n">
         <v>4.2</v>
       </c>
       <c r="G3" t="n">
-        <v>3850</v>
+        <v>6750</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Kapiva Original Himalayan Shilajit Resin</t>
+          <t>Kapiva Original Himalayan Shilajit/Shilajeet Resin 40g |Super Saver Pack| 250mg/Serving | For Energy, Endurance &amp; Vitality | 160 Servings | 100% Ayurvedic</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>500</v>
+        <v>1648</v>
       </c>
       <c r="F4" t="n">
         <v>4.1</v>
       </c>
       <c r="G4" t="n">
-        <v>10194</v>
+        <v>3221</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -602,7 +602,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -624,17 +624,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Kapiva Shilajit Gold Capsules</t>
+          <t>Kapiva Shilajit/Shilajeet Gold 60 Capsules | Contains 24 Carat Gold | For Stamina, Muscle Growth &amp; Energy | Ashwagandha, Gokshura, Safed Musali &amp; Other Action Herbs &amp; 100% Ayurvedic</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>500</v>
+        <v>1199</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>1255</v>
+        <v>3853</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -670,17 +670,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kapiva Original Himalayan Shilajit/Shilajeet Resin 20g | 250mg/Serving | For Energy, Endurance &amp; Vitality | 80 Servings | 100% Ayurvedic</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>500</v>
+        <v>699</v>
       </c>
       <c r="F6" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>10210</v>
+        <v>10159</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -716,17 +716,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Kapiva Get Slim Juice Healthy Weight Management</t>
+          <t>Kapiva Get Slim Juice - Healthy Weight Management Through 12 Ayurvedic Herbs Aids Metabolism and Digestion - 1L</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>500</v>
+        <v>479</v>
       </c>
       <c r="F7" t="n">
         <v>3.8</v>
       </c>
       <c r="G7" t="n">
-        <v>833</v>
+        <v>9778</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Kapiva Get Slim Juice</t>
+          <t>Kapiva Get Slim Juice (2L) Bottle,Pack| Healthy Weight Management Through 12 Ayurvedic Herbs | Aids Metabolism and Digestion - Super Saver Pack of 2</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>500</v>
+        <v>978</v>
       </c>
       <c r="F8" t="n">
         <v>3.9</v>
       </c>
       <c r="G8" t="n">
-        <v>9835</v>
+        <v>1119</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -808,17 +808,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Kapiva Plant Protein | 25g Protein Per Scoop, Chocolate | With Vitamins &amp;amp; Minerals | Pea protein Isolate - 1Kg : Amazon.in: Health &amp;amp; Personal Care</t>
+          <t>Kapiva Plant Protein | 25g Protein Per Scoop, Chocolate | With Vitamins &amp; Minerals | Pea protein Isolate - 1Kg</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>500</v>
+        <v>1779</v>
       </c>
       <c r="F9" t="n">
         <v>3.9</v>
       </c>
       <c r="G9" t="n">
-        <v>244</v>
+        <v>758</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -854,17 +854,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Kapiva Certified A2 Gir Cow Ghee 500ML | Traditional Vedic Bilona Method | Grassfed, Pure &amp;amp; Healthy | Curd-Churned | Premium Glass Bottle | 100% Natural &amp;amp; Lab-Tested | Rich in Nutrition : Amazon.in: Grocery &amp;amp; Gourmet Foods</t>
+          <t>Kapiva Certified A2 Gir Cow Ghee 500ML | Traditional Vedic Bilona Method | Grassfed, Pure &amp; Healthy | Curd-Churned | Premium Glass Bottle | Lab-Tested | Rich in Nutrition</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>500</v>
+        <v>744</v>
       </c>
       <c r="F10" t="n">
         <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>2599</v>
+        <v>1380</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -900,17 +900,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kapiva Skin Foods Glow Mix Ayurvedic Collagen Powder</t>
+          <t>Kapiva Skin Foods Glow Mix | Ayurvedic Skin Supplement, Collagen Powder | Skincare for Glowing &amp; Healthy Skin (30 Sachets)</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>500</v>
+        <v>888</v>
       </c>
       <c r="F11" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="G11" t="n">
-        <v>784</v>
+        <v>2468</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -946,17 +946,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kapiva Hair Care Juice for Hair Growth &amp;amp; Hair Fall Control</t>
+          <t>Kapiva Hair Care Juice (2L) | For Hair Growth &amp; Hair Fall Control | 100% Ayurvedic Hair Care with Amla, Noni, Bhringraj and Ashwagandha - Super Saver Pack of 2</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>500</v>
+        <v>1452</v>
       </c>
       <c r="F12" t="n">
         <v>3.9</v>
       </c>
       <c r="G12" t="n">
-        <v>1607</v>
+        <v>199</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -992,17 +992,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Kapiva Pure Aloe Vera Skin Gel 500g For Face &amp;amp; Hair | Hydrating, Moisturizing, Soothing Skin | Multipurpose Gel : Amazon.in: Beauty</t>
+          <t>Kapiva Pure Aloe Vera Skin Gel 500g For Face &amp; Hair | Hydrating, Moisturizing, Soothing Skin | Multipurpose Gel</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>500</v>
+        <v>349</v>
       </c>
       <c r="F13" t="n">
         <v>4.2</v>
       </c>
       <c r="G13" t="n">
-        <v>16399</v>
+        <v>6221</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>success</t>
         </is>
       </c>
     </row>

</xml_diff>